<commit_message>
Refaz fechamento: teto 4% últ. compra / 6% média hist. e 1 arquivo por OL
Nova regra de aceitação (substitui 5%/10%-zerado): preço aprovado se
≤ últ. compra × 1,04 OU ≤ média histórica × 1,06. Pedidos finais: 902
itens, R$ 73.005,42 em 9 distribuidores. OLs voltam a 1 arquivo por OL
(25 arquivos, 968 itens), substituindo a lista única. Verificado:
nenhum item de OL nos pedidos.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VLivvbyTHZf5HaiMxTfGPo
</commit_message>
<xml_diff>
--- a/cotacoes/2026-09-08/fechamento/PEDIDO_AT_SUPLEMENTOS_09-09-2026.xlsx
+++ b/cotacoes/2026-09-08/fechamento/PEDIDO_AT_SUPLEMENTOS_09-09-2026.xlsx
@@ -465,7 +465,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q46"/>
+  <dimension ref="A1:Q40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -576,30 +576,30 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>673351</v>
+        <v>597651</v>
       </c>
       <c r="B2" s="2" t="inlineStr"/>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>7899941207714</t>
+          <t>7896311763269</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>100% WHEY DOUBLE TASTY MAXTITANIUM BAUNI</t>
+          <t>AMINO BCAA INTEGRALMEDICA 90 CAPS</t>
         </is>
       </c>
       <c r="E2" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F2" s="4" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="G2" s="4" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="H2" s="5" t="n">
-        <v>130</v>
+        <v>45</v>
       </c>
       <c r="I2" s="5">
         <f>G2*H2</f>
@@ -610,13 +610,13 @@
         <v/>
       </c>
       <c r="K2" s="5" t="n">
-        <v>119.98</v>
+        <v>45.25</v>
       </c>
       <c r="L2" s="5" t="n">
-        <v>106.99</v>
+        <v>38.06</v>
       </c>
       <c r="M2" s="5" t="n">
-        <v>115.65</v>
+        <v>42.85333333333333</v>
       </c>
       <c r="N2" s="6">
         <f>J2/M2-1</f>
@@ -628,37 +628,37 @@
       </c>
       <c r="P2" s="2" t="inlineStr">
         <is>
-          <t>REAJUSTE +8.4% (aceito, lim 10% zerado)</t>
+          <t>OK (≤ últ. compra)</t>
         </is>
       </c>
       <c r="Q2" s="2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
-        <v>597651</v>
+        <v>9703</v>
       </c>
       <c r="B3" s="2" t="inlineStr"/>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>7896311763269</t>
+          <t>7898920041592</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>AMINO BCAA INTEGRALMEDICA 90 CAPS</t>
+          <t>BCAA 2400MG MAX TITANIUM 100 CAPS</t>
         </is>
       </c>
       <c r="E3" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F3" s="4" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="G3" s="4" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="H3" s="5" t="n">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="I3" s="5">
         <f>G3*H3</f>
@@ -669,13 +669,13 @@
         <v/>
       </c>
       <c r="K3" s="5" t="n">
-        <v>45.25</v>
+        <v>48.7</v>
       </c>
       <c r="L3" s="5" t="n">
-        <v>38.06</v>
+        <v>42.64</v>
       </c>
       <c r="M3" s="5" t="n">
-        <v>42.85333333333333</v>
+        <v>44.66</v>
       </c>
       <c r="N3" s="6">
         <f>J3/M3-1</f>
@@ -694,17 +694,17 @@
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
-        <v>9703</v>
+        <v>666601</v>
       </c>
       <c r="B4" s="2" t="inlineStr"/>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>7898920041592</t>
+          <t>7898755180336</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>BCAA 2400MG MAX TITANIUM 100 CAPS</t>
+          <t>BOLD BAR BANOFFEE D/12 UN 60G CX C/12</t>
         </is>
       </c>
       <c r="E4" s="4" t="n">
@@ -717,7 +717,7 @@
         <v>1</v>
       </c>
       <c r="H4" s="5" t="n">
-        <v>48</v>
+        <v>11.35</v>
       </c>
       <c r="I4" s="5">
         <f>G4*H4</f>
@@ -728,13 +728,13 @@
         <v/>
       </c>
       <c r="K4" s="5" t="n">
-        <v>48.7</v>
+        <v>141.12</v>
       </c>
       <c r="L4" s="5" t="n">
-        <v>42.64</v>
+        <v>141.12</v>
       </c>
       <c r="M4" s="5" t="n">
-        <v>44.66</v>
+        <v>141.12</v>
       </c>
       <c r="N4" s="6">
         <f>J4/M4-1</f>
@@ -749,21 +749,25 @@
           <t>OK (≤ últ. compra)</t>
         </is>
       </c>
-      <c r="Q4" s="2" t="inlineStr"/>
+      <c r="Q4" s="2" t="inlineStr">
+        <is>
+          <t>conferir emb.</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
-        <v>666601</v>
+        <v>609311</v>
       </c>
       <c r="B5" s="2" t="inlineStr"/>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>7898755180336</t>
+          <t>609963966240</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>BOLD BAR BANOFFEE D/12 UN 60G CX C/12</t>
+          <t>BOLD BAR THIN COOKIES CREAM 40G</t>
         </is>
       </c>
       <c r="E5" s="4" t="n">
@@ -776,7 +780,7 @@
         <v>1</v>
       </c>
       <c r="H5" s="5" t="n">
-        <v>11.35</v>
+        <v>7.65</v>
       </c>
       <c r="I5" s="5">
         <f>G5*H5</f>
@@ -787,13 +791,13 @@
         <v/>
       </c>
       <c r="K5" s="5" t="n">
-        <v>141.12</v>
+        <v>7.59</v>
       </c>
       <c r="L5" s="5" t="n">
-        <v>141.12</v>
+        <v>7.59</v>
       </c>
       <c r="M5" s="5" t="n">
-        <v>141.12</v>
+        <v>7.59</v>
       </c>
       <c r="N5" s="6">
         <f>J5/M5-1</f>
@@ -805,28 +809,24 @@
       </c>
       <c r="P5" s="2" t="inlineStr">
         <is>
-          <t>OK (≤ menor hist.)</t>
-        </is>
-      </c>
-      <c r="Q5" s="2" t="inlineStr">
-        <is>
-          <t>conferir emb.</t>
-        </is>
-      </c>
+          <t>REAJUSTE +0.8% vs últ. (≤4%)</t>
+        </is>
+      </c>
+      <c r="Q5" s="2" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
-        <v>609311</v>
+        <v>609321</v>
       </c>
       <c r="B6" s="2" t="inlineStr"/>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>609963966240</t>
+          <t>609963966288</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>BOLD BAR THIN COOKIES CREAM 40G</t>
+          <t>BOLD BAR THIN TRUFA DE MORANGO 40G D/12</t>
         </is>
       </c>
       <c r="E6" s="4" t="n">
@@ -868,24 +868,24 @@
       </c>
       <c r="P6" s="2" t="inlineStr">
         <is>
-          <t>REAJUSTE +0.8% (aceito, lim 10% zerado)</t>
+          <t>REAJUSTE +0.8% vs últ. (≤4%)</t>
         </is>
       </c>
       <c r="Q6" s="2" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
-        <v>609321</v>
+        <v>602181</v>
       </c>
       <c r="B7" s="2" t="inlineStr"/>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>609963966288</t>
+          <t>7897104920784</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>BOLD BAR THIN TRUFA DE MORANGO 40G D/12</t>
+          <t>COLAGENO HIDRO VERISOL C/ ACIDO HIALURONICO BODYACTION LAR/ACEROLA 200G</t>
         </is>
       </c>
       <c r="E7" s="4" t="n">
@@ -898,7 +898,7 @@
         <v>1</v>
       </c>
       <c r="H7" s="5" t="n">
-        <v>7.65</v>
+        <v>55</v>
       </c>
       <c r="I7" s="5">
         <f>G7*H7</f>
@@ -909,13 +909,13 @@
         <v/>
       </c>
       <c r="K7" s="5" t="n">
-        <v>7.59</v>
+        <v>54.9</v>
       </c>
       <c r="L7" s="5" t="n">
-        <v>7.59</v>
+        <v>54.9</v>
       </c>
       <c r="M7" s="5" t="n">
-        <v>7.59</v>
+        <v>54.9</v>
       </c>
       <c r="N7" s="6">
         <f>J7/M7-1</f>
@@ -927,24 +927,24 @@
       </c>
       <c r="P7" s="2" t="inlineStr">
         <is>
-          <t>REAJUSTE +0.8% (aceito, lim 10% zerado)</t>
+          <t>REAJUSTE +0.2% vs últ. (≤4%)</t>
         </is>
       </c>
       <c r="Q7" s="2" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
-        <v>602181</v>
+        <v>597681</v>
       </c>
       <c r="B8" s="2" t="inlineStr"/>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>7897104920784</t>
+          <t>7897104907396</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>COLAGENO HIDRO VERISOL C/ ACIDO HIALURONICO BODYACTION LAR/ACEROLA 200G</t>
+          <t>COLAGENO VERISOL COM ACIDO HIALURONICO BODYACTION 90CAP</t>
         </is>
       </c>
       <c r="E8" s="4" t="n">
@@ -968,13 +968,13 @@
         <v/>
       </c>
       <c r="K8" s="5" t="n">
-        <v>54.9</v>
+        <v>55.51</v>
       </c>
       <c r="L8" s="5" t="n">
-        <v>54.9</v>
+        <v>55.51</v>
       </c>
       <c r="M8" s="5" t="n">
-        <v>54.9</v>
+        <v>55.51</v>
       </c>
       <c r="N8" s="6">
         <f>J8/M8-1</f>
@@ -986,24 +986,24 @@
       </c>
       <c r="P8" s="2" t="inlineStr">
         <is>
-          <t>REAJUSTE +0.2% (aceito, lim 10% zerado)</t>
+          <t>OK (≤ últ. compra)</t>
         </is>
       </c>
       <c r="Q8" s="2" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
-        <v>597681</v>
+        <v>650841</v>
       </c>
       <c r="B9" s="2" t="inlineStr"/>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>7897104907396</t>
+          <t>7898583668457</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>COLAGENO VERISOL COM ACIDO HIALURONICO BODYACTION 90CAP</t>
+          <t>CREATINA FTW 1KG</t>
         </is>
       </c>
       <c r="E9" s="4" t="n">
@@ -1016,7 +1016,7 @@
         <v>1</v>
       </c>
       <c r="H9" s="5" t="n">
-        <v>55</v>
+        <v>142</v>
       </c>
       <c r="I9" s="5">
         <f>G9*H9</f>
@@ -1027,13 +1027,13 @@
         <v/>
       </c>
       <c r="K9" s="5" t="n">
-        <v>55.51</v>
+        <v>161.42</v>
       </c>
       <c r="L9" s="5" t="n">
-        <v>55.51</v>
+        <v>161.42</v>
       </c>
       <c r="M9" s="5" t="n">
-        <v>55.51</v>
+        <v>161.42</v>
       </c>
       <c r="N9" s="6">
         <f>J9/M9-1</f>
@@ -1045,37 +1045,37 @@
       </c>
       <c r="P9" s="2" t="inlineStr">
         <is>
-          <t>OK (≤ menor hist.)</t>
+          <t>OK (≤ últ. compra)</t>
         </is>
       </c>
       <c r="Q9" s="2" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
-        <v>650841</v>
+        <v>630451</v>
       </c>
       <c r="B10" s="2" t="inlineStr"/>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>7898583668457</t>
+          <t>7896311708314</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>CREATINA FTW 1KG</t>
+          <t>CREATINA INTEGRALMEDICA HARDCORE RELOAD 300G</t>
         </is>
       </c>
       <c r="E10" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F10" s="4" t="n">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="G10" s="4" t="n">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="H10" s="5" t="n">
-        <v>142</v>
+        <v>46</v>
       </c>
       <c r="I10" s="5">
         <f>G10*H10</f>
@@ -1086,13 +1086,13 @@
         <v/>
       </c>
       <c r="K10" s="5" t="n">
-        <v>161.42</v>
+        <v>46.54</v>
       </c>
       <c r="L10" s="5" t="n">
-        <v>161.42</v>
+        <v>36.1</v>
       </c>
       <c r="M10" s="5" t="n">
-        <v>161.42</v>
+        <v>39.58000000000001</v>
       </c>
       <c r="N10" s="6">
         <f>J10/M10-1</f>
@@ -1104,37 +1104,37 @@
       </c>
       <c r="P10" s="2" t="inlineStr">
         <is>
-          <t>OK (≤ menor hist.)</t>
+          <t>OK (≤ últ. compra)</t>
         </is>
       </c>
       <c r="Q10" s="2" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
-        <v>630451</v>
+        <v>597701</v>
       </c>
       <c r="B11" s="2" t="inlineStr"/>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>7896311708314</t>
+          <t>7896311763498</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>CREATINA INTEGRALMEDICA HARDCORE RELOAD 300G</t>
+          <t>CREATINA INTEGRALMEDICA PT 150G</t>
         </is>
       </c>
       <c r="E11" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F11" s="4" t="n">
-        <v>30</v>
+        <v>17</v>
       </c>
       <c r="G11" s="4" t="n">
-        <v>30</v>
+        <v>17</v>
       </c>
       <c r="H11" s="5" t="n">
-        <v>46</v>
+        <v>28</v>
       </c>
       <c r="I11" s="5">
         <f>G11*H11</f>
@@ -1145,13 +1145,13 @@
         <v/>
       </c>
       <c r="K11" s="5" t="n">
-        <v>46.54</v>
+        <v>28.42</v>
       </c>
       <c r="L11" s="5" t="n">
-        <v>36.1</v>
+        <v>17.59</v>
       </c>
       <c r="M11" s="5" t="n">
-        <v>39.58000000000001</v>
+        <v>21.2</v>
       </c>
       <c r="N11" s="6">
         <f>J11/M11-1</f>
@@ -1170,30 +1170,30 @@
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
-        <v>597701</v>
+        <v>672991</v>
       </c>
       <c r="B12" s="2" t="inlineStr"/>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>7896311763498</t>
+          <t>7896311709083</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>CREATINA INTEGRALMEDICA PT 150G</t>
+          <t>CREATINA WHITE 60 CAPS</t>
         </is>
       </c>
       <c r="E12" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F12" s="4" t="n">
-        <v>17</v>
+        <v>4</v>
       </c>
       <c r="G12" s="4" t="n">
-        <v>17</v>
+        <v>4</v>
       </c>
       <c r="H12" s="5" t="n">
-        <v>28</v>
+        <v>21</v>
       </c>
       <c r="I12" s="5">
         <f>G12*H12</f>
@@ -1204,13 +1204,13 @@
         <v/>
       </c>
       <c r="K12" s="5" t="n">
-        <v>28.42</v>
+        <v>21.78</v>
       </c>
       <c r="L12" s="5" t="n">
-        <v>17.59</v>
+        <v>16.28</v>
       </c>
       <c r="M12" s="5" t="n">
-        <v>21.2</v>
+        <v>18.16666666666667</v>
       </c>
       <c r="N12" s="6">
         <f>J12/M12-1</f>
@@ -1229,17 +1229,17 @@
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
-        <v>672991</v>
+        <v>597731</v>
       </c>
       <c r="B13" s="2" t="inlineStr"/>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>7896311709083</t>
+          <t>7898708731394</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>CREATINA WHITE 60 CAPS</t>
+          <t>CREATINE TURBO BLACKSKULL 150G</t>
         </is>
       </c>
       <c r="E13" s="4" t="n">
@@ -1252,7 +1252,7 @@
         <v>4</v>
       </c>
       <c r="H13" s="5" t="n">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="I13" s="5">
         <f>G13*H13</f>
@@ -1263,13 +1263,13 @@
         <v/>
       </c>
       <c r="K13" s="5" t="n">
-        <v>21.78</v>
+        <v>36.15</v>
       </c>
       <c r="L13" s="5" t="n">
-        <v>16.28</v>
+        <v>36.15</v>
       </c>
       <c r="M13" s="5" t="n">
-        <v>18.16666666666667</v>
+        <v>36.15</v>
       </c>
       <c r="N13" s="6">
         <f>J13/M13-1</f>
@@ -1288,17 +1288,17 @@
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
-        <v>597731</v>
+        <v>635321</v>
       </c>
       <c r="B14" s="2" t="inlineStr"/>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t>7898708731394</t>
+          <t>7898957433544</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>CREATINE TURBO BLACKSKULL 150G</t>
+          <t>CREATINY MONOHYDRATE CANIBALINC 300G</t>
         </is>
       </c>
       <c r="E14" s="4" t="n">
@@ -1311,7 +1311,7 @@
         <v>4</v>
       </c>
       <c r="H14" s="5" t="n">
-        <v>25</v>
+        <v>38</v>
       </c>
       <c r="I14" s="5">
         <f>G14*H14</f>
@@ -1322,13 +1322,13 @@
         <v/>
       </c>
       <c r="K14" s="5" t="n">
-        <v>36.15</v>
+        <v>38.84</v>
       </c>
       <c r="L14" s="5" t="n">
-        <v>36.15</v>
+        <v>38.84</v>
       </c>
       <c r="M14" s="5" t="n">
-        <v>36.15</v>
+        <v>38.84</v>
       </c>
       <c r="N14" s="6">
         <f>J14/M14-1</f>
@@ -1340,37 +1340,37 @@
       </c>
       <c r="P14" s="2" t="inlineStr">
         <is>
-          <t>OK (≤ menor hist.)</t>
+          <t>OK (≤ últ. compra)</t>
         </is>
       </c>
       <c r="Q14" s="2" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
-        <v>635321</v>
+        <v>657881</v>
       </c>
       <c r="B15" s="2" t="inlineStr"/>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>7898957433544</t>
+          <t>7896311774845</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>CREATINY MONOHYDRATE CANIBALINC 300G</t>
+          <t>DARK BAR DARKNESS CREME DE COCO C/ CASTANHA D/08 90G CX C/8</t>
         </is>
       </c>
       <c r="E15" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F15" s="4" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="G15" s="4" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="H15" s="5" t="n">
-        <v>38</v>
+        <v>14</v>
       </c>
       <c r="I15" s="5">
         <f>G15*H15</f>
@@ -1381,13 +1381,13 @@
         <v/>
       </c>
       <c r="K15" s="5" t="n">
-        <v>38.84</v>
+        <v>95</v>
       </c>
       <c r="L15" s="5" t="n">
-        <v>38.84</v>
+        <v>95</v>
       </c>
       <c r="M15" s="5" t="n">
-        <v>38.84</v>
+        <v>95</v>
       </c>
       <c r="N15" s="6">
         <f>J15/M15-1</f>
@@ -1399,24 +1399,28 @@
       </c>
       <c r="P15" s="2" t="inlineStr">
         <is>
-          <t>OK (≤ menor hist.)</t>
-        </is>
-      </c>
-      <c r="Q15" s="2" t="inlineStr"/>
+          <t>OK (≤ últ. compra)</t>
+        </is>
+      </c>
+      <c r="Q15" s="2" t="inlineStr">
+        <is>
+          <t>conferir emb.</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
-        <v>657881</v>
+        <v>638251</v>
       </c>
       <c r="B16" s="2" t="inlineStr"/>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t>7896311774845</t>
+          <t>7899598008740</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>DARK BAR DARKNESS CREME DE COCO C/ CASTANHA D/08 90G CX C/8</t>
+          <t>DIABO VERDE FTW INSANO ENERGETICO 150G</t>
         </is>
       </c>
       <c r="E16" s="4" t="n">
@@ -1429,7 +1433,7 @@
         <v>1</v>
       </c>
       <c r="H16" s="5" t="n">
-        <v>14</v>
+        <v>58</v>
       </c>
       <c r="I16" s="5">
         <f>G16*H16</f>
@@ -1440,13 +1444,13 @@
         <v/>
       </c>
       <c r="K16" s="5" t="n">
-        <v>95</v>
+        <v>56.91</v>
       </c>
       <c r="L16" s="5" t="n">
-        <v>95</v>
+        <v>56.91</v>
       </c>
       <c r="M16" s="5" t="n">
-        <v>95</v>
+        <v>56.91</v>
       </c>
       <c r="N16" s="6">
         <f>J16/M16-1</f>
@@ -1458,28 +1462,24 @@
       </c>
       <c r="P16" s="2" t="inlineStr">
         <is>
-          <t>OK (≤ menor hist.)</t>
-        </is>
-      </c>
-      <c r="Q16" s="2" t="inlineStr">
-        <is>
-          <t>conferir emb.</t>
-        </is>
-      </c>
+          <t>REAJUSTE +1.9% vs últ. (≤4%)</t>
+        </is>
+      </c>
+      <c r="Q16" s="2" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
-        <v>638251</v>
+        <v>602171</v>
       </c>
       <c r="B17" s="2" t="inlineStr"/>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>7899598008740</t>
+          <t>7898583666279</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>DIABO VERDE FTW INSANO ENERGETICO 150G</t>
+          <t>DIABO VERDE FTW INSANO FRUTAS AMARELAS 150G</t>
         </is>
       </c>
       <c r="E17" s="4" t="n">
@@ -1503,13 +1503,13 @@
         <v/>
       </c>
       <c r="K17" s="5" t="n">
-        <v>56.91</v>
+        <v>59.9</v>
       </c>
       <c r="L17" s="5" t="n">
         <v>56.91</v>
       </c>
       <c r="M17" s="5" t="n">
-        <v>56.91</v>
+        <v>57.90666666666667</v>
       </c>
       <c r="N17" s="6">
         <f>J17/M17-1</f>
@@ -1521,24 +1521,24 @@
       </c>
       <c r="P17" s="2" t="inlineStr">
         <is>
-          <t>REAJUSTE +1.9% (aceito, lim 10% zerado)</t>
+          <t>OK (≤ últ. compra)</t>
         </is>
       </c>
       <c r="Q17" s="2" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="2" t="n">
-        <v>602171</v>
+        <v>602161</v>
       </c>
       <c r="B18" s="2" t="inlineStr"/>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t>7898583666279</t>
+          <t>7899598008733</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>DIABO VERDE FTW INSANO FRUTAS AMARELAS 150G</t>
+          <t>DIABO VERDE FTW INSANO MACA VERDE 150G</t>
         </is>
       </c>
       <c r="E18" s="4" t="n">
@@ -1587,17 +1587,17 @@
     </row>
     <row r="19">
       <c r="A19" s="2" t="n">
-        <v>602161</v>
+        <v>638261</v>
       </c>
       <c r="B19" s="2" t="inlineStr"/>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t>7899598008733</t>
+          <t>7898583666538</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>DIABO VERDE FTW INSANO MACA VERDE 150G</t>
+          <t>DIABO VERDE FTW PRE WORKOUT LIMAO 150</t>
         </is>
       </c>
       <c r="E19" s="4" t="n">
@@ -1624,10 +1624,10 @@
         <v>59.9</v>
       </c>
       <c r="L19" s="5" t="n">
-        <v>56.91</v>
+        <v>58.79</v>
       </c>
       <c r="M19" s="5" t="n">
-        <v>57.90666666666667</v>
+        <v>59.53</v>
       </c>
       <c r="N19" s="6">
         <f>J19/M19-1</f>
@@ -1646,17 +1646,17 @@
     </row>
     <row r="20">
       <c r="A20" s="2" t="n">
-        <v>638261</v>
+        <v>655871</v>
       </c>
       <c r="B20" s="2" t="inlineStr"/>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t>7898583666538</t>
+          <t>7899598025495</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>DIABO VERDE FTW PRE WORKOUT LIMAO 150</t>
+          <t>DIABO VERDE PRE WORKOUT FTW FRUTAS VERMELHAS 150G</t>
         </is>
       </c>
       <c r="E20" s="4" t="n">
@@ -1683,10 +1683,10 @@
         <v>59.9</v>
       </c>
       <c r="L20" s="5" t="n">
-        <v>58.79</v>
+        <v>56.91</v>
       </c>
       <c r="M20" s="5" t="n">
-        <v>59.53</v>
+        <v>57.90666666666667</v>
       </c>
       <c r="N20" s="6">
         <f>J20/M20-1</f>
@@ -1698,37 +1698,37 @@
       </c>
       <c r="P20" s="2" t="inlineStr">
         <is>
-          <t>OK (≤ menor hist.)</t>
+          <t>OK (≤ últ. compra)</t>
         </is>
       </c>
       <c r="Q20" s="2" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="2" t="n">
-        <v>655871</v>
+        <v>30103</v>
       </c>
       <c r="B21" s="2" t="inlineStr"/>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t>7899598025495</t>
+          <t>07897104909604</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>DIABO VERDE PRE WORKOUT FTW FRUTAS VERMELHAS 150G</t>
+          <t>ENERGEL BLACK BODYACTION ACAI/GUARAN 30G</t>
         </is>
       </c>
       <c r="E21" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F21" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G21" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H21" s="5" t="n">
-        <v>58</v>
+        <v>2.96</v>
       </c>
       <c r="I21" s="5">
         <f>G21*H21</f>
@@ -1739,13 +1739,13 @@
         <v/>
       </c>
       <c r="K21" s="5" t="n">
-        <v>59.9</v>
+        <v>2.93</v>
       </c>
       <c r="L21" s="5" t="n">
-        <v>56.91</v>
+        <v>2.93</v>
       </c>
       <c r="M21" s="5" t="n">
-        <v>57.90666666666667</v>
+        <v>2.93</v>
       </c>
       <c r="N21" s="6">
         <f>J21/M21-1</f>
@@ -1757,34 +1757,34 @@
       </c>
       <c r="P21" s="2" t="inlineStr">
         <is>
-          <t>OK (≤ últ. compra)</t>
+          <t>REAJUSTE +1.0% vs últ. (≤4%)</t>
         </is>
       </c>
       <c r="Q21" s="2" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="2" t="n">
-        <v>30103</v>
+        <v>602151</v>
       </c>
       <c r="B22" s="2" t="inlineStr"/>
       <c r="C22" s="3" t="inlineStr">
         <is>
-          <t>07897104909604</t>
+          <t>7897104910242</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>ENERGEL BLACK BODYACTION ACAI/GUARAN 30G</t>
+          <t>ENERGEL BLACK BODYACTION FRUTAS VERMELHAS 30G D/10</t>
         </is>
       </c>
       <c r="E22" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F22" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G22" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H22" s="5" t="n">
         <v>2.96</v>
@@ -1798,13 +1798,13 @@
         <v/>
       </c>
       <c r="K22" s="5" t="n">
-        <v>2.93</v>
+        <v>23.3</v>
       </c>
       <c r="L22" s="5" t="n">
-        <v>2.93</v>
+        <v>23.3</v>
       </c>
       <c r="M22" s="5" t="n">
-        <v>2.93</v>
+        <v>23.3</v>
       </c>
       <c r="N22" s="6">
         <f>J22/M22-1</f>
@@ -1816,24 +1816,28 @@
       </c>
       <c r="P22" s="2" t="inlineStr">
         <is>
-          <t>REAJUSTE +1.0% (aceito, lim 10% zerado)</t>
-        </is>
-      </c>
-      <c r="Q22" s="2" t="inlineStr"/>
+          <t>OK (≤ últ. compra)</t>
+        </is>
+      </c>
+      <c r="Q22" s="2" t="inlineStr">
+        <is>
+          <t>conferir emb.</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="n">
-        <v>602151</v>
+        <v>29403</v>
       </c>
       <c r="B23" s="2" t="inlineStr"/>
       <c r="C23" s="3" t="inlineStr">
         <is>
-          <t>7897104910242</t>
+          <t>7897104928445</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>ENERGEL BLACK BODYACTION FRUTAS VERMELHAS 30G D/10</t>
+          <t>ENERGEL BLACK BODYACTION LARAN/ACERO 30G</t>
         </is>
       </c>
       <c r="E23" s="4" t="n">
@@ -1857,13 +1861,13 @@
         <v/>
       </c>
       <c r="K23" s="5" t="n">
-        <v>23.3</v>
+        <v>3.18</v>
       </c>
       <c r="L23" s="5" t="n">
-        <v>23.3</v>
+        <v>3.18</v>
       </c>
       <c r="M23" s="5" t="n">
-        <v>23.3</v>
+        <v>3.18</v>
       </c>
       <c r="N23" s="6">
         <f>J23/M23-1</f>
@@ -1875,28 +1879,24 @@
       </c>
       <c r="P23" s="2" t="inlineStr">
         <is>
-          <t>OK (≤ menor hist.)</t>
-        </is>
-      </c>
-      <c r="Q23" s="2" t="inlineStr">
-        <is>
-          <t>conferir emb.</t>
-        </is>
-      </c>
+          <t>OK (≤ últ. compra)</t>
+        </is>
+      </c>
+      <c r="Q23" s="2" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="2" t="n">
-        <v>29403</v>
+        <v>666581</v>
       </c>
       <c r="B24" s="2" t="inlineStr"/>
       <c r="C24" s="3" t="inlineStr">
         <is>
-          <t>7897104928445</t>
+          <t>7897104926229</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>ENERGEL BLACK BODYACTION LARAN/ACERO 30G</t>
+          <t>ENERGEL BLACK BODYACTION UVA D/10 30G CX C/10</t>
         </is>
       </c>
       <c r="E24" s="4" t="n">
@@ -1920,13 +1920,13 @@
         <v/>
       </c>
       <c r="K24" s="5" t="n">
-        <v>3.18</v>
+        <v>2.97</v>
       </c>
       <c r="L24" s="5" t="n">
-        <v>3.18</v>
+        <v>2.97</v>
       </c>
       <c r="M24" s="5" t="n">
-        <v>3.18</v>
+        <v>2.97</v>
       </c>
       <c r="N24" s="6">
         <f>J24/M24-1</f>
@@ -1938,24 +1938,24 @@
       </c>
       <c r="P24" s="2" t="inlineStr">
         <is>
-          <t>OK (≤ menor hist.)</t>
+          <t>OK (≤ últ. compra)</t>
         </is>
       </c>
       <c r="Q24" s="2" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="2" t="n">
-        <v>666581</v>
+        <v>597751</v>
       </c>
       <c r="B25" s="2" t="inlineStr"/>
       <c r="C25" s="3" t="inlineStr">
         <is>
-          <t>7897104926229</t>
+          <t>7897104905200</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>ENERGEL BLACK BODYACTION UVA D/10 30G CX C/10</t>
+          <t>HARDMASS 1800 BODYACTION CHOCOLATE PC 3K</t>
         </is>
       </c>
       <c r="E25" s="4" t="n">
@@ -1968,7 +1968,7 @@
         <v>1</v>
       </c>
       <c r="H25" s="5" t="n">
-        <v>2.96</v>
+        <v>85</v>
       </c>
       <c r="I25" s="5">
         <f>G25*H25</f>
@@ -1979,13 +1979,13 @@
         <v/>
       </c>
       <c r="K25" s="5" t="n">
-        <v>2.97</v>
+        <v>82.42</v>
       </c>
       <c r="L25" s="5" t="n">
-        <v>2.97</v>
+        <v>82.42</v>
       </c>
       <c r="M25" s="5" t="n">
-        <v>2.97</v>
+        <v>82.42</v>
       </c>
       <c r="N25" s="6">
         <f>J25/M25-1</f>
@@ -1997,24 +1997,24 @@
       </c>
       <c r="P25" s="2" t="inlineStr">
         <is>
-          <t>OK (≤ menor hist.)</t>
+          <t>REAJUSTE +3.1% vs últ. (≤4%)</t>
         </is>
       </c>
       <c r="Q25" s="2" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="2" t="n">
-        <v>597751</v>
+        <v>661421</v>
       </c>
       <c r="B26" s="2" t="inlineStr"/>
       <c r="C26" s="3" t="inlineStr">
         <is>
-          <t>7897104905200</t>
+          <t>7897104905194</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>HARDMASS 1800 BODYACTION CHOCOLATE PC 3K</t>
+          <t>HARDMASS 1800 BODYACTION MORANGO PC 3KG</t>
         </is>
       </c>
       <c r="E26" s="4" t="n">
@@ -2056,24 +2056,24 @@
       </c>
       <c r="P26" s="2" t="inlineStr">
         <is>
-          <t>REAJUSTE +3.1% (aceito, lim 10% zerado)</t>
+          <t>REAJUSTE +3.1% vs últ. (≤4%)</t>
         </is>
       </c>
       <c r="Q26" s="2" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="2" t="n">
-        <v>661421</v>
+        <v>673371</v>
       </c>
       <c r="B27" s="2" t="inlineStr"/>
       <c r="C27" s="3" t="inlineStr">
         <is>
-          <t>7897104905194</t>
+          <t>7898920041318</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>HARDMASS 1800 BODYACTION MORANGO PC 3KG</t>
+          <t>MASS TITANIUM 17500 BAUNILHA 3KG</t>
         </is>
       </c>
       <c r="E27" s="4" t="n">
@@ -2086,7 +2086,7 @@
         <v>1</v>
       </c>
       <c r="H27" s="5" t="n">
-        <v>85</v>
+        <v>93</v>
       </c>
       <c r="I27" s="5">
         <f>G27*H27</f>
@@ -2097,13 +2097,13 @@
         <v/>
       </c>
       <c r="K27" s="5" t="n">
-        <v>82.42</v>
+        <v>93.20999999999999</v>
       </c>
       <c r="L27" s="5" t="n">
-        <v>82.42</v>
+        <v>86.75</v>
       </c>
       <c r="M27" s="5" t="n">
-        <v>82.42</v>
+        <v>88.90333333333332</v>
       </c>
       <c r="N27" s="6">
         <f>J27/M27-1</f>
@@ -2115,24 +2115,24 @@
       </c>
       <c r="P27" s="2" t="inlineStr">
         <is>
-          <t>REAJUSTE +3.1% (aceito, lim 10% zerado)</t>
+          <t>OK (≤ últ. compra)</t>
         </is>
       </c>
       <c r="Q27" s="2" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="2" t="n">
-        <v>673371</v>
+        <v>638291</v>
       </c>
       <c r="B28" s="2" t="inlineStr"/>
       <c r="C28" s="3" t="inlineStr">
         <is>
-          <t>7898920041318</t>
+          <t>7897104926243</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>MASS TITANIUM 17500 BAUNILHA 3KG</t>
+          <t>NUCLEAR RUSH BODYACTION LARANJA 100G</t>
         </is>
       </c>
       <c r="E28" s="4" t="n">
@@ -2145,7 +2145,7 @@
         <v>1</v>
       </c>
       <c r="H28" s="5" t="n">
-        <v>93</v>
+        <v>40</v>
       </c>
       <c r="I28" s="5">
         <f>G28*H28</f>
@@ -2156,13 +2156,13 @@
         <v/>
       </c>
       <c r="K28" s="5" t="n">
-        <v>93.20999999999999</v>
+        <v>38.16</v>
       </c>
       <c r="L28" s="5" t="n">
-        <v>86.75</v>
+        <v>38.16</v>
       </c>
       <c r="M28" s="5" t="n">
-        <v>88.90333333333332</v>
+        <v>38.16</v>
       </c>
       <c r="N28" s="6">
         <f>J28/M28-1</f>
@@ -2174,37 +2174,37 @@
       </c>
       <c r="P28" s="2" t="inlineStr">
         <is>
-          <t>OK (≤ últ. compra)</t>
+          <t>REAJUSTE +4.8% vs média (≤6%)</t>
         </is>
       </c>
       <c r="Q28" s="2" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="2" t="n">
-        <v>661351</v>
+        <v>673321</v>
       </c>
       <c r="B29" s="2" t="inlineStr"/>
       <c r="C29" s="3" t="inlineStr">
         <is>
-          <t>7896311773657</t>
+          <t>7897104925444</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>MY WHEY INTEGRALMEDICA MORANGO PT 900G</t>
+          <t>NUCLEAR RUSH GEL BODYACTION FRUTAS V 25G</t>
         </is>
       </c>
       <c r="E29" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F29" s="4" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="G29" s="4" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="H29" s="5" t="n">
-        <v>117</v>
+        <v>2.99</v>
       </c>
       <c r="I29" s="5">
         <f>G29*H29</f>
@@ -2215,13 +2215,13 @@
         <v/>
       </c>
       <c r="K29" s="5" t="n">
-        <v>110.68</v>
+        <v>2.99</v>
       </c>
       <c r="L29" s="5" t="n">
-        <v>87.3</v>
+        <v>2.75</v>
       </c>
       <c r="M29" s="5" t="n">
-        <v>99.73</v>
+        <v>2.91</v>
       </c>
       <c r="N29" s="6">
         <f>J29/M29-1</f>
@@ -2233,24 +2233,24 @@
       </c>
       <c r="P29" s="2" t="inlineStr">
         <is>
-          <t>REAJUSTE +5.7% (aceito, lim 10% zerado)</t>
+          <t>OK (≤ últ. compra)</t>
         </is>
       </c>
       <c r="Q29" s="2" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="2" t="n">
-        <v>638291</v>
+        <v>638311</v>
       </c>
       <c r="B30" s="2" t="inlineStr"/>
       <c r="C30" s="3" t="inlineStr">
         <is>
-          <t>7897104926243</t>
+          <t>7893596226427</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>NUCLEAR RUSH BODYACTION LARANJA 100G</t>
+          <t>PANIC PRE WORKOUT ADAPTOGEN UVA 150G</t>
         </is>
       </c>
       <c r="E30" s="4" t="n">
@@ -2263,7 +2263,7 @@
         <v>1</v>
       </c>
       <c r="H30" s="5" t="n">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="I30" s="5">
         <f>G30*H30</f>
@@ -2274,13 +2274,13 @@
         <v/>
       </c>
       <c r="K30" s="5" t="n">
-        <v>38.16</v>
+        <v>62.61</v>
       </c>
       <c r="L30" s="5" t="n">
-        <v>38.16</v>
+        <v>62.61</v>
       </c>
       <c r="M30" s="5" t="n">
-        <v>38.16</v>
+        <v>62.60999999999999</v>
       </c>
       <c r="N30" s="6">
         <f>J30/M30-1</f>
@@ -2292,37 +2292,37 @@
       </c>
       <c r="P30" s="2" t="inlineStr">
         <is>
-          <t>REAJUSTE +4.8% (aceito, lim 10% zerado)</t>
+          <t>OK (≤ últ. compra)</t>
         </is>
       </c>
       <c r="Q30" s="2" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="2" t="n">
-        <v>673321</v>
+        <v>672961</v>
       </c>
       <c r="B31" s="2" t="inlineStr"/>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>7897104925444</t>
+          <t>7896311778041</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>NUCLEAR RUSH GEL BODYACTION FRUTAS V 25G</t>
+          <t>PROTEIN CRISP INTEGRAL OVOMALTIN 45G</t>
         </is>
       </c>
       <c r="E31" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F31" s="4" t="n">
-        <v>22</v>
+        <v>6</v>
       </c>
       <c r="G31" s="4" t="n">
-        <v>22</v>
+        <v>6</v>
       </c>
       <c r="H31" s="5" t="n">
-        <v>2.99</v>
+        <v>8</v>
       </c>
       <c r="I31" s="5">
         <f>G31*H31</f>
@@ -2333,13 +2333,13 @@
         <v/>
       </c>
       <c r="K31" s="5" t="n">
-        <v>2.99</v>
+        <v>8.050000000000001</v>
       </c>
       <c r="L31" s="5" t="n">
-        <v>2.75</v>
+        <v>6.23</v>
       </c>
       <c r="M31" s="5" t="n">
-        <v>2.91</v>
+        <v>6.973333333333334</v>
       </c>
       <c r="N31" s="6">
         <f>J31/M31-1</f>
@@ -2358,30 +2358,30 @@
     </row>
     <row r="32">
       <c r="A32" s="2" t="n">
-        <v>673331</v>
+        <v>646181</v>
       </c>
       <c r="B32" s="2" t="inlineStr"/>
       <c r="C32" s="3" t="inlineStr">
         <is>
-          <t>7897104925437</t>
+          <t>7899941203211</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>NUCLEAR RUSH GEL BODYACTION GUARANA 25G</t>
+          <t>PV - HORUS MAX TITANIUM MACA VERDE POTE 150G</t>
         </is>
       </c>
       <c r="E32" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F32" s="4" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="G32" s="4" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="H32" s="5" t="n">
-        <v>2.99</v>
+        <v>59</v>
       </c>
       <c r="I32" s="5">
         <f>G32*H32</f>
@@ -2392,13 +2392,13 @@
         <v/>
       </c>
       <c r="K32" s="5" t="n">
-        <v>2.75</v>
+        <v>63.61</v>
       </c>
       <c r="L32" s="5" t="n">
-        <v>2.75</v>
+        <v>63.61</v>
       </c>
       <c r="M32" s="5" t="n">
-        <v>2.75</v>
+        <v>63.60999999999999</v>
       </c>
       <c r="N32" s="6">
         <f>J32/M32-1</f>
@@ -2410,24 +2410,24 @@
       </c>
       <c r="P32" s="2" t="inlineStr">
         <is>
-          <t>REAJUSTE +8.7% (aceito, lim 10% zerado)</t>
+          <t>OK (≤ últ. compra)</t>
         </is>
       </c>
       <c r="Q32" s="2" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="2" t="n">
-        <v>638311</v>
+        <v>635411</v>
       </c>
       <c r="B33" s="2" t="inlineStr"/>
       <c r="C33" s="3" t="inlineStr">
         <is>
-          <t>7893596226427</t>
+          <t>7896311775439</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>PANIC PRE WORKOUT ADAPTOGEN UVA 150G</t>
+          <t>REFIL CREAMASS INTEGRALMEDICA CHOCOLATE 3KG</t>
         </is>
       </c>
       <c r="E33" s="4" t="n">
@@ -2440,7 +2440,7 @@
         <v>1</v>
       </c>
       <c r="H33" s="5" t="n">
-        <v>60</v>
+        <v>106</v>
       </c>
       <c r="I33" s="5">
         <f>G33*H33</f>
@@ -2451,13 +2451,13 @@
         <v/>
       </c>
       <c r="K33" s="5" t="n">
-        <v>62.61</v>
+        <v>106.26</v>
       </c>
       <c r="L33" s="5" t="n">
-        <v>62.61</v>
+        <v>79.20999999999999</v>
       </c>
       <c r="M33" s="5" t="n">
-        <v>62.60999999999999</v>
+        <v>89.10666666666667</v>
       </c>
       <c r="N33" s="6">
         <f>J33/M33-1</f>
@@ -2469,37 +2469,37 @@
       </c>
       <c r="P33" s="2" t="inlineStr">
         <is>
-          <t>OK (≤ menor hist.)</t>
+          <t>OK (≤ últ. compra)</t>
         </is>
       </c>
       <c r="Q33" s="2" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="2" t="n">
-        <v>602041</v>
+        <v>661501</v>
       </c>
       <c r="B34" s="2" t="inlineStr"/>
       <c r="C34" s="3" t="inlineStr">
         <is>
-          <t>7898939072617</t>
+          <t>7898626448343</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>PASTA DE AMENDOIM POWER1ONE CROCANTE 1,005KG (L)</t>
+          <t>REFIL ISOLATE PROTEIN MIX PROFIT BAUNILHA 900G</t>
         </is>
       </c>
       <c r="E34" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F34" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G34" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H34" s="5" t="n">
-        <v>27</v>
+        <v>71</v>
       </c>
       <c r="I34" s="5">
         <f>G34*H34</f>
@@ -2510,13 +2510,13 @@
         <v/>
       </c>
       <c r="K34" s="5" t="n">
-        <v>25.81</v>
+        <v>71.40000000000001</v>
       </c>
       <c r="L34" s="5" t="n">
-        <v>20.81</v>
+        <v>71.40000000000001</v>
       </c>
       <c r="M34" s="5" t="n">
-        <v>22.47666666666666</v>
+        <v>71.40000000000001</v>
       </c>
       <c r="N34" s="6">
         <f>J34/M34-1</f>
@@ -2528,37 +2528,37 @@
       </c>
       <c r="P34" s="2" t="inlineStr">
         <is>
-          <t>REAJUSTE +4.6% (aceito, lim 10% zerado)</t>
+          <t>OK (≤ últ. compra)</t>
         </is>
       </c>
       <c r="Q34" s="2" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" s="2" t="n">
-        <v>672961</v>
+        <v>30003</v>
       </c>
       <c r="B35" s="2" t="inlineStr"/>
       <c r="C35" s="3" t="inlineStr">
         <is>
-          <t>7896311778041</t>
+          <t>7896311778072</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>PROTEIN CRISP INTEGRAL OVOMALTIN 45G</t>
+          <t>REFIL NUTRIWHEY INTEGRAL MORANGO 1,2KG</t>
         </is>
       </c>
       <c r="E35" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F35" s="4" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="G35" s="4" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="H35" s="5" t="n">
-        <v>8</v>
+        <v>85</v>
       </c>
       <c r="I35" s="5">
         <f>G35*H35</f>
@@ -2569,13 +2569,13 @@
         <v/>
       </c>
       <c r="K35" s="5" t="n">
-        <v>8.050000000000001</v>
+        <v>85.67</v>
       </c>
       <c r="L35" s="5" t="n">
-        <v>6.23</v>
+        <v>85.67</v>
       </c>
       <c r="M35" s="5" t="n">
-        <v>6.973333333333334</v>
+        <v>85.67</v>
       </c>
       <c r="N35" s="6">
         <f>J35/M35-1</f>
@@ -2594,30 +2594,30 @@
     </row>
     <row r="36">
       <c r="A36" s="2" t="n">
-        <v>646181</v>
+        <v>29703</v>
       </c>
       <c r="B36" s="2" t="inlineStr"/>
       <c r="C36" s="3" t="inlineStr">
         <is>
-          <t>7899941203211</t>
+          <t>7898626449623</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>PV - HORUS MAX TITANIUM MACA VERDE POTE 150G</t>
+          <t>RF ISOLATE PROTEIN MIX PROFIT LEITE 900G</t>
         </is>
       </c>
       <c r="E36" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F36" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G36" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H36" s="5" t="n">
-        <v>59</v>
+        <v>71</v>
       </c>
       <c r="I36" s="5">
         <f>G36*H36</f>
@@ -2628,13 +2628,13 @@
         <v/>
       </c>
       <c r="K36" s="5" t="n">
-        <v>63.61</v>
+        <v>71.40000000000001</v>
       </c>
       <c r="L36" s="5" t="n">
-        <v>63.61</v>
+        <v>71.40000000000001</v>
       </c>
       <c r="M36" s="5" t="n">
-        <v>63.60999999999999</v>
+        <v>71.40000000000001</v>
       </c>
       <c r="N36" s="6">
         <f>J36/M36-1</f>
@@ -2646,24 +2646,24 @@
       </c>
       <c r="P36" s="2" t="inlineStr">
         <is>
-          <t>OK (≤ menor hist.)</t>
+          <t>OK (≤ últ. compra)</t>
         </is>
       </c>
       <c r="Q36" s="2" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" s="2" t="n">
-        <v>618891</v>
+        <v>661461</v>
       </c>
       <c r="B37" s="2" t="inlineStr"/>
       <c r="C37" s="3" t="inlineStr">
         <is>
-          <t>7899941202023</t>
+          <t>7898708731516</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>REFIL 100% WHEY MAX TITANIUM COOKIES E CREAM 900G</t>
+          <t>THERMO FLAME CAVEIRAPRETA 120 TABLETES</t>
         </is>
       </c>
       <c r="E37" s="4" t="n">
@@ -2676,7 +2676,7 @@
         <v>1</v>
       </c>
       <c r="H37" s="5" t="n">
-        <v>139</v>
+        <v>22</v>
       </c>
       <c r="I37" s="5">
         <f>G37*H37</f>
@@ -2687,13 +2687,13 @@
         <v/>
       </c>
       <c r="K37" s="5" t="n">
-        <v>127.93</v>
+        <v>39.65</v>
       </c>
       <c r="L37" s="5" t="n">
-        <v>101.11</v>
+        <v>39.65</v>
       </c>
       <c r="M37" s="5" t="n">
-        <v>115.3566666666667</v>
+        <v>39.65</v>
       </c>
       <c r="N37" s="6">
         <f>J37/M37-1</f>
@@ -2705,380 +2705,26 @@
       </c>
       <c r="P37" s="2" t="inlineStr">
         <is>
-          <t>REAJUSTE +8.7% (aceito, lim 10% zerado)</t>
+          <t>OK (≤ últ. compra)</t>
         </is>
       </c>
       <c r="Q37" s="2" t="inlineStr"/>
     </row>
     <row r="38">
-      <c r="A38" s="2" t="n">
-        <v>643321</v>
-      </c>
-      <c r="B38" s="2" t="inlineStr"/>
-      <c r="C38" s="3" t="inlineStr">
-        <is>
-          <t>7899941201712</t>
-        </is>
-      </c>
-      <c r="D38" s="2" t="inlineStr">
-        <is>
-          <t>REFIL 100% WHEY MAX TITANIUM MORANGO  900G</t>
-        </is>
-      </c>
-      <c r="E38" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="F38" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="G38" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="H38" s="5" t="n">
-        <v>139</v>
-      </c>
-      <c r="I38" s="5">
-        <f>G38*H38</f>
-        <v/>
-      </c>
-      <c r="J38" s="5">
-        <f>H38/E38</f>
-        <v/>
-      </c>
-      <c r="K38" s="5" t="n">
-        <v>127.93</v>
-      </c>
-      <c r="L38" s="5" t="n">
-        <v>101.11</v>
-      </c>
-      <c r="M38" s="5" t="n">
-        <v>115.3566666666667</v>
-      </c>
-      <c r="N38" s="6">
-        <f>J38/M38-1</f>
-        <v/>
-      </c>
-      <c r="O38" s="6">
-        <f>J38/K38-1</f>
-        <v/>
-      </c>
-      <c r="P38" s="2" t="inlineStr">
-        <is>
-          <t>REAJUSTE +8.7% (aceito, lim 10% zerado)</t>
-        </is>
-      </c>
-      <c r="Q38" s="2" t="inlineStr"/>
-    </row>
-    <row r="39">
-      <c r="A39" s="2" t="n">
-        <v>635411</v>
-      </c>
-      <c r="B39" s="2" t="inlineStr"/>
-      <c r="C39" s="3" t="inlineStr">
-        <is>
-          <t>7896311775439</t>
-        </is>
-      </c>
-      <c r="D39" s="2" t="inlineStr">
-        <is>
-          <t>REFIL CREAMASS INTEGRALMEDICA CHOCOLATE 3KG</t>
-        </is>
-      </c>
-      <c r="E39" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="F39" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="G39" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="H39" s="5" t="n">
-        <v>106</v>
-      </c>
-      <c r="I39" s="5">
-        <f>G39*H39</f>
-        <v/>
-      </c>
-      <c r="J39" s="5">
-        <f>H39/E39</f>
-        <v/>
-      </c>
-      <c r="K39" s="5" t="n">
-        <v>106.26</v>
-      </c>
-      <c r="L39" s="5" t="n">
-        <v>79.20999999999999</v>
-      </c>
-      <c r="M39" s="5" t="n">
-        <v>89.10666666666667</v>
-      </c>
-      <c r="N39" s="6">
-        <f>J39/M39-1</f>
-        <v/>
-      </c>
-      <c r="O39" s="6">
-        <f>J39/K39-1</f>
-        <v/>
-      </c>
-      <c r="P39" s="2" t="inlineStr">
-        <is>
-          <t>OK (≤ últ. compra)</t>
-        </is>
-      </c>
-      <c r="Q39" s="2" t="inlineStr"/>
+      <c r="D38" s="7" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="I38" s="8">
+        <f>SUM(I2:I37)</f>
+        <v/>
+      </c>
     </row>
     <row r="40">
-      <c r="A40" s="2" t="n">
-        <v>661501</v>
-      </c>
-      <c r="B40" s="2" t="inlineStr"/>
-      <c r="C40" s="3" t="inlineStr">
-        <is>
-          <t>7898626448343</t>
-        </is>
-      </c>
-      <c r="D40" s="2" t="inlineStr">
-        <is>
-          <t>REFIL ISOLATE PROTEIN MIX PROFIT BAUNILHA 900G</t>
-        </is>
-      </c>
-      <c r="E40" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="F40" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="G40" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="H40" s="5" t="n">
-        <v>71</v>
-      </c>
-      <c r="I40" s="5">
-        <f>G40*H40</f>
-        <v/>
-      </c>
-      <c r="J40" s="5">
-        <f>H40/E40</f>
-        <v/>
-      </c>
-      <c r="K40" s="5" t="n">
-        <v>71.40000000000001</v>
-      </c>
-      <c r="L40" s="5" t="n">
-        <v>71.40000000000001</v>
-      </c>
-      <c r="M40" s="5" t="n">
-        <v>71.40000000000001</v>
-      </c>
-      <c r="N40" s="6">
-        <f>J40/M40-1</f>
-        <v/>
-      </c>
-      <c r="O40" s="6">
-        <f>J40/K40-1</f>
-        <v/>
-      </c>
-      <c r="P40" s="2" t="inlineStr">
-        <is>
-          <t>OK (≤ menor hist.)</t>
-        </is>
-      </c>
-      <c r="Q40" s="2" t="inlineStr"/>
-    </row>
-    <row r="41">
-      <c r="A41" s="2" t="n">
-        <v>30003</v>
-      </c>
-      <c r="B41" s="2" t="inlineStr"/>
-      <c r="C41" s="3" t="inlineStr">
-        <is>
-          <t>7896311778072</t>
-        </is>
-      </c>
-      <c r="D41" s="2" t="inlineStr">
-        <is>
-          <t>REFIL NUTRIWHEY INTEGRAL MORANGO 1,2KG</t>
-        </is>
-      </c>
-      <c r="E41" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="F41" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="G41" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="H41" s="5" t="n">
-        <v>85</v>
-      </c>
-      <c r="I41" s="5">
-        <f>G41*H41</f>
-        <v/>
-      </c>
-      <c r="J41" s="5">
-        <f>H41/E41</f>
-        <v/>
-      </c>
-      <c r="K41" s="5" t="n">
-        <v>85.67</v>
-      </c>
-      <c r="L41" s="5" t="n">
-        <v>85.67</v>
-      </c>
-      <c r="M41" s="5" t="n">
-        <v>85.67</v>
-      </c>
-      <c r="N41" s="6">
-        <f>J41/M41-1</f>
-        <v/>
-      </c>
-      <c r="O41" s="6">
-        <f>J41/K41-1</f>
-        <v/>
-      </c>
-      <c r="P41" s="2" t="inlineStr">
-        <is>
-          <t>OK (≤ menor hist.)</t>
-        </is>
-      </c>
-      <c r="Q41" s="2" t="inlineStr"/>
-    </row>
-    <row r="42">
-      <c r="A42" s="2" t="n">
-        <v>29703</v>
-      </c>
-      <c r="B42" s="2" t="inlineStr"/>
-      <c r="C42" s="3" t="inlineStr">
-        <is>
-          <t>7898626449623</t>
-        </is>
-      </c>
-      <c r="D42" s="2" t="inlineStr">
-        <is>
-          <t>RF ISOLATE PROTEIN MIX PROFIT LEITE 900G</t>
-        </is>
-      </c>
-      <c r="E42" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="F42" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="G42" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="H42" s="5" t="n">
-        <v>71</v>
-      </c>
-      <c r="I42" s="5">
-        <f>G42*H42</f>
-        <v/>
-      </c>
-      <c r="J42" s="5">
-        <f>H42/E42</f>
-        <v/>
-      </c>
-      <c r="K42" s="5" t="n">
-        <v>71.40000000000001</v>
-      </c>
-      <c r="L42" s="5" t="n">
-        <v>71.40000000000001</v>
-      </c>
-      <c r="M42" s="5" t="n">
-        <v>71.40000000000001</v>
-      </c>
-      <c r="N42" s="6">
-        <f>J42/M42-1</f>
-        <v/>
-      </c>
-      <c r="O42" s="6">
-        <f>J42/K42-1</f>
-        <v/>
-      </c>
-      <c r="P42" s="2" t="inlineStr">
-        <is>
-          <t>OK (≤ menor hist.)</t>
-        </is>
-      </c>
-      <c r="Q42" s="2" t="inlineStr"/>
-    </row>
-    <row r="43">
-      <c r="A43" s="2" t="n">
-        <v>661461</v>
-      </c>
-      <c r="B43" s="2" t="inlineStr"/>
-      <c r="C43" s="3" t="inlineStr">
-        <is>
-          <t>7898708731516</t>
-        </is>
-      </c>
-      <c r="D43" s="2" t="inlineStr">
-        <is>
-          <t>THERMO FLAME CAVEIRAPRETA 120 TABLETES</t>
-        </is>
-      </c>
-      <c r="E43" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="F43" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="G43" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="H43" s="5" t="n">
-        <v>22</v>
-      </c>
-      <c r="I43" s="5">
-        <f>G43*H43</f>
-        <v/>
-      </c>
-      <c r="J43" s="5">
-        <f>H43/E43</f>
-        <v/>
-      </c>
-      <c r="K43" s="5" t="n">
-        <v>39.65</v>
-      </c>
-      <c r="L43" s="5" t="n">
-        <v>39.65</v>
-      </c>
-      <c r="M43" s="5" t="n">
-        <v>39.65</v>
-      </c>
-      <c r="N43" s="6">
-        <f>J43/M43-1</f>
-        <v/>
-      </c>
-      <c r="O43" s="6">
-        <f>J43/K43-1</f>
-        <v/>
-      </c>
-      <c r="P43" s="2" t="inlineStr">
-        <is>
-          <t>OK (≤ menor hist.)</t>
-        </is>
-      </c>
-      <c r="Q43" s="2" t="inlineStr"/>
-    </row>
-    <row r="44">
-      <c r="D44" s="7" t="inlineStr">
-        <is>
-          <t>TOTAL</t>
-        </is>
-      </c>
-      <c r="I44" s="8">
-        <f>SUM(I2:I43)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="9" t="inlineStr">
-        <is>
-          <t>Pedido FINAL AT_SUPLEMENTOS — cotação 08/09/2026 (fechada 09/09). Somente itens aprovados: preço até 5% acima da referência (últ. compra; sem ela, menor histórico), 10% quando o item está zerado. 'Qtd pedido' na embalagem do fornecedor.</t>
+      <c r="A40" s="9" t="inlineStr">
+        <is>
+          <t>Pedido FINAL AT_SUPLEMENTOS — cotação 08/09/2026 (fechada 09/09). Somente itens aprovados: teto de reajuste de 4% sobre a última compra OU 6% sobre a média histórica (3/6/12m). 'Qtd pedido' na embalagem do fornecedor.</t>
         </is>
       </c>
     </row>

</xml_diff>